<commit_message>
Fix test case generation for Leave module + SCRUM-45 end-to-end verification
</commit_message>
<xml_diff>
--- a/artifacts/SCRUM-45/SCRUM-45_TestCases.xlsx
+++ b/artifacts/SCRUM-45/SCRUM-45_TestCases.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="60">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -63,25 +63,48 @@
     <t>The application loads successfully and is accessible.</t>
   </si>
   <si>
+    <t>Test passed successfully.</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>UI</t>
+  </si>
+  <si>
+    <t>Automated</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>High</t>
-  </si>
-  <si>
-    <t>UI</t>
-  </si>
-  <si>
-    <t>Automated</t>
-  </si>
-  <si>
-    <t>Not Run</t>
-  </si>
-  <si>
     <t>TC_UI_02</t>
   </si>
   <si>
     <t>Verify: User can navigate to the *Leave* module.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Launch the OrangeHRM application and log in as Admin.
+2. Navigate to My Info.
+3. Verify the page loads without errors.
+4. From the top menu bar, click "Leave".
+5. Verify the Leave module loads and displays the Leave List or My Leave view.
+6. Verify the page shows leave options like "Apply", "My Leave", or "Entitlements".</t>
+  </si>
+  <si>
+    <t>The leave request is submitted successfully.</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>TC_UI_03</t>
+  </si>
+  <si>
+    <t>Verify: User can locate an existing leave request that is eligible for modification.</t>
   </si>
   <si>
     <t xml:space="preserve">1. Launch the OrangeHRM application and log in as Admin.
@@ -93,22 +116,25 @@
 7. Verify the leave request is submitted successfully.</t>
   </si>
   <si>
-    <t>The leave request is submitted successfully.</t>
-  </si>
-  <si>
-    <t>Medium</t>
-  </si>
-  <si>
-    <t>TC_UI_03</t>
-  </si>
-  <si>
-    <t>Verify: User can locate an existing leave request that is eligible for modification.</t>
-  </si>
-  <si>
     <t>TC_UI_04</t>
   </si>
   <si>
     <t>Verify: User can edit the leave request details (e.g., leave dates or leave type).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Launch the OrangeHRM application and log in as Admin.
+2. Navigate to My Info.
+3. Verify the page loads without errors.
+4. From the top menu bar, click "Leave".
+5. Click "My Leave" to view the leave list/calendar.
+6. Locate an existing leave request from the list that is eligible for modification (Pending or Cancelled status).
+7. Click the "Edit" icon or action for the existing leave request.
+8. Modify the leave details (e.g., change dates, leave type, or add comments).
+9. Click "Save" or "Update" to apply the changes.
+10. Verify the updated leave details are reflected in the leave list.</t>
+  </si>
+  <si>
+    <t>The existing leave request is updated successfully.</t>
   </si>
   <si>
     <t>TC_UI_05</t>
@@ -131,7 +157,7 @@
 6. Verify the expected result is displayed.</t>
   </si>
   <si>
-    <t>The action for "A success confirmation message is displayed." completes successfully with the expected result displayed.</t>
+    <t>A success confirmation message is displayed.</t>
   </si>
   <si>
     <t>TC_UI_07</t>
@@ -171,6 +197,9 @@
     <t>The page content is rendered and visible.</t>
   </si>
   <si>
+    <t>Not Run</t>
+  </si>
+  <si>
     <t>TC_API_01</t>
   </si>
   <si>
@@ -206,7 +235,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -217,6 +246,10 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF22C55E"/>
     </font>
   </fonts>
   <fills count="3">
@@ -267,7 +300,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -690,30 +723,30 @@
         <v>20</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" ht="115" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" ht="100" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>16</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>18</v>
@@ -725,30 +758,30 @@
         <v>20</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" ht="115" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>16</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>18</v>
@@ -760,30 +793,30 @@
         <v>20</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" ht="115" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" ht="160" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>16</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>18</v>
@@ -795,30 +828,30 @@
         <v>20</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" ht="115" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" ht="160" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>16</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>18</v>
@@ -830,30 +863,30 @@
         <v>20</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" ht="100" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>16</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>18</v>
@@ -865,30 +898,30 @@
         <v>20</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" ht="115" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" ht="160" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>16</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>18</v>
@@ -900,30 +933,30 @@
         <v>20</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" ht="100" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>16</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>18</v>
@@ -935,30 +968,30 @@
         <v>20</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" ht="55" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>18</v>
@@ -967,36 +1000,36 @@
         <v>19</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" ht="55" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>16</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>19</v>
@@ -1005,46 +1038,46 @@
         <v>20</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" ht="55" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>19</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>